<commit_message>
Migrate config references to record keys
</commit_message>
<xml_diff>
--- a/examples/humanpark/data/Configs.xlsx
+++ b/examples/humanpark/data/Configs.xlsx
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="820" uniqueCount="749">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="754">
   <si>
     <t>id</t>
   </si>
@@ -2649,6 +2649,21 @@
   </si>
   <si>
     <t>Gene_LingHuoE|Gene_FaGuangQi</t>
+  </si>
+  <si>
+    <t>@Gene_SimpleDivision|@Gene_Chloroplast|@Gene_Flagellum|@Gene_LvShi</t>
+  </si>
+  <si>
+    <t>@Gene_LingHuoE|@Gene_FaGuangQi</t>
+  </si>
+  <si>
+    <t>@Gene_TanHuangJiRou</t>
+  </si>
+  <si>
+    <t>@Gene_DuCiXiBao</t>
+  </si>
+  <si>
+    <t>@Gene_Genius</t>
   </si>
 </sst>
 </file>
@@ -3523,12 +3538,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02C66289-10C9-4243-BA3F-16CAB580811F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{02C66289-10C9-4243-BA3F-16CAB580811F}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:H20"/>
-  <sheetFormatPr defaultColWidth="14" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="14" defaultRowHeight="12.75" ns3:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
@@ -3538,7 +3553,7 @@
     <col min="8" max="8" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" ns3:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>746</v>
       </c>
@@ -3564,7 +3579,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" ns3:dyDescent="0.2">
       <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
@@ -3572,7 +3587,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>9</v>
+        <v>751</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>10</v>
@@ -3587,7 +3602,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" ns3:dyDescent="0.2">
       <c r="B3" s="3" t="s">
         <v>12</v>
       </c>
@@ -3595,7 +3610,7 @@
         <v>8</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>13</v>
+        <v>752</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>14</v>
@@ -3610,7 +3625,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" ns3:dyDescent="0.2">
       <c r="B4" s="3" t="s">
         <v>15</v>
       </c>
@@ -3618,7 +3633,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>16</v>
+        <v>753</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>17</v>
@@ -3633,89 +3648,89 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" ns3:dyDescent="0.2">
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" ns3:dyDescent="0.2">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" ns3:dyDescent="0.2">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" ns3:dyDescent="0.2">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" ns3:dyDescent="0.2">
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" ns3:dyDescent="0.2">
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" ns3:dyDescent="0.2">
       <c r="B11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" ns3:dyDescent="0.2">
       <c r="E12" s="3"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" ns3:dyDescent="0.2">
       <c r="B13" s="3"/>
       <c r="D13" s="3"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" ns3:dyDescent="0.2">
       <c r="E14" s="3"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" ns3:dyDescent="0.2">
       <c r="D15" s="3"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" ns3:dyDescent="0.2">
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:5" ns3:dyDescent="0.2">
       <c r="B17" s="3"/>
       <c r="E17" s="3"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:5" ns3:dyDescent="0.2">
       <c r="D18" s="3"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:5" ns3:dyDescent="0.2">
       <c r="E19" s="3"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:5" ns3:dyDescent="0.2">
       <c r="B20" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <drawing ns4:id="rId1"/>
+  <legacyDrawing ns4:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD5DD13A-E6DE-4484-8F70-F8E417AF8006}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{AD5DD13A-E6DE-4484-8F70-F8E417AF8006}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultColWidth="14" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="14" defaultRowHeight="12.75" ns3:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
@@ -3729,7 +3744,7 @@
     <col min="11" max="11" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ns3:dyDescent="0.2">
       <c r="A1" s="71" t="s">
         <v>746</v>
       </c>
@@ -3752,7 +3767,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" ns3:dyDescent="0.2">
       <c r="B2" s="3" t="s">
         <v>734</v>
       </c>
@@ -3769,10 +3784,10 @@
         <v>736</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>747</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ns3:dyDescent="0.2">
       <c r="B3" s="3" t="s">
         <v>737</v>
       </c>
@@ -3786,7 +3801,7 @@
         <v>500</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
     </row>
   </sheetData>
@@ -9253,12 +9268,12 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0957BDD-BE50-4E05-8C6D-72BFAE44711C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns4="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{F0957BDD-BE50-4E05-8C6D-72BFAE44711C}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:R149"/>
-  <sheetFormatPr defaultColWidth="14" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="14" defaultRowHeight="12.75" ns3:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -9269,7 +9284,7 @@
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" ns3:dyDescent="0.2">
       <c r="A1" s="51" t="s">
         <v>746</v>
       </c>
@@ -9295,7 +9310,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" ns3:dyDescent="0.2">
       <c r="A2" s="53" t="s">
         <v>537</v>
       </c>
@@ -9319,7 +9334,7 @@
       <c r="Q2" s="56"/>
       <c r="R2" s="56"/>
     </row>
-    <row r="3" spans="1:18" ht="51" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" ht="51" ns3:dyDescent="0.2">
       <c r="B3" s="11" t="s">
         <v>539</v>
       </c>
@@ -9337,7 +9352,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:18" ht="25.5" ns3:dyDescent="0.2">
       <c r="B4" s="11" t="s">
         <v>542</v>
       </c>
@@ -9355,7 +9370,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" ht="33" customHeight="1" ns3:dyDescent="0.2">
       <c r="A5" s="12"/>
       <c r="B5" s="17" t="s">
         <v>545</v>
@@ -9385,7 +9400,7 @@
       <c r="Q5" s="12"/>
       <c r="R5" s="12"/>
     </row>
-    <row r="6" spans="1:18" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" ht="33" customHeight="1" ns3:dyDescent="0.2">
       <c r="A6" s="17"/>
       <c r="B6" s="17" t="s">
         <v>547</v>
@@ -9415,7 +9430,7 @@
       <c r="Q6" s="12"/>
       <c r="R6" s="12"/>
     </row>
-    <row r="7" spans="1:18" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" ht="33" customHeight="1" ns3:dyDescent="0.2">
       <c r="A7" s="17"/>
       <c r="B7" s="17" t="s">
         <v>550</v>
@@ -9445,7 +9460,7 @@
       <c r="Q7" s="12"/>
       <c r="R7" s="12"/>
     </row>
-    <row r="8" spans="1:18" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:18" ht="33" customHeight="1" ns3:dyDescent="0.2">
       <c r="A8" s="11"/>
       <c r="B8" s="11" t="s">
         <v>553</v>
@@ -9475,7 +9490,7 @@
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:18" ns3:dyDescent="0.2">
       <c r="A9" s="53" t="s">
         <v>537</v>
       </c>
@@ -9499,7 +9514,7 @@
       <c r="Q9" s="56"/>
       <c r="R9" s="56"/>
     </row>
-    <row r="10" spans="1:18" ht="45.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" ht="45.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A10" s="17"/>
       <c r="B10" s="17" t="s">
         <v>557</v>
@@ -9529,7 +9544,7 @@
       <c r="Q10" s="12"/>
       <c r="R10" s="12"/>
     </row>
-    <row r="11" spans="1:18" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" ht="25.5" ns3:dyDescent="0.2">
       <c r="A11" s="11"/>
       <c r="B11" s="17" t="s">
         <v>560</v>
@@ -9548,7 +9563,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:18" ns3:dyDescent="0.2">
       <c r="A12" s="11"/>
       <c r="B12" s="17" t="s">
         <v>563</v>
@@ -9567,7 +9582,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:18" ns3:dyDescent="0.2">
       <c r="A13" s="53" t="s">
         <v>537</v>
       </c>
@@ -9591,7 +9606,7 @@
       <c r="Q13" s="56"/>
       <c r="R13" s="56"/>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:18" ns3:dyDescent="0.2">
       <c r="A14" s="11"/>
       <c r="B14" s="17" t="s">
         <v>567</v>
@@ -9610,7 +9625,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A15" s="11"/>
       <c r="B15" s="17" t="s">
         <v>570</v>
@@ -9640,7 +9655,7 @@
       <c r="Q15" s="3"/>
       <c r="R15" s="3"/>
     </row>
-    <row r="16" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A16" s="11"/>
       <c r="B16" s="17" t="s">
         <v>573</v>
@@ -9670,7 +9685,7 @@
       <c r="Q16" s="3"/>
       <c r="R16" s="3"/>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:18" ns3:dyDescent="0.2">
       <c r="A17" s="11"/>
       <c r="B17" s="17" t="s">
         <v>576</v>
@@ -9690,7 +9705,7 @@
       </c>
       <c r="H17" s="3"/>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:18" ns3:dyDescent="0.2">
       <c r="A18" s="11"/>
       <c r="B18" s="17" t="s">
         <v>579</v>
@@ -9710,7 +9725,7 @@
       </c>
       <c r="H18" s="3"/>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:18" ns3:dyDescent="0.2">
       <c r="A19" s="11"/>
       <c r="B19" s="11" t="s">
         <v>582</v>
@@ -9731,7 +9746,7 @@
       <c r="I19" s="11"/>
       <c r="J19" s="3"/>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:18" ns3:dyDescent="0.2">
       <c r="A20" s="60"/>
       <c r="B20" s="60" t="s">
         <v>585</v>
@@ -9761,7 +9776,7 @@
       <c r="Q20" s="62"/>
       <c r="R20" s="62"/>
     </row>
-    <row r="21" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A21" s="60"/>
       <c r="B21" s="60" t="s">
         <v>588</v>
@@ -9791,7 +9806,7 @@
       <c r="Q21" s="62"/>
       <c r="R21" s="62"/>
     </row>
-    <row r="22" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A22" s="53" t="s">
         <v>537</v>
       </c>
@@ -9815,7 +9830,7 @@
       <c r="Q22" s="56"/>
       <c r="R22" s="56"/>
     </row>
-    <row r="23" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A23" s="17"/>
       <c r="B23" s="17" t="s">
         <v>592</v>
@@ -9845,7 +9860,7 @@
       <c r="Q23" s="12"/>
       <c r="R23" s="12"/>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:18" ns3:dyDescent="0.2">
       <c r="A24" s="60"/>
       <c r="B24" s="60" t="s">
         <v>595</v>
@@ -9875,7 +9890,7 @@
       <c r="Q24" s="62"/>
       <c r="R24" s="62"/>
     </row>
-    <row r="25" spans="1:18" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:18" ht="33" customHeight="1" ns3:dyDescent="0.2">
       <c r="A25" s="60"/>
       <c r="B25" s="60" t="s">
         <v>598</v>
@@ -9905,7 +9920,7 @@
       <c r="Q25" s="62"/>
       <c r="R25" s="62"/>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:18" ns3:dyDescent="0.2">
       <c r="A26" s="60"/>
       <c r="B26" s="60" t="s">
         <v>601</v>
@@ -9935,7 +9950,7 @@
       <c r="Q26" s="62"/>
       <c r="R26" s="62"/>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:18" ns3:dyDescent="0.2">
       <c r="A27" s="60"/>
       <c r="B27" s="60" t="s">
         <v>604</v>
@@ -9965,7 +9980,7 @@
       <c r="Q27" s="62"/>
       <c r="R27" s="62"/>
     </row>
-    <row r="28" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A28" s="60"/>
       <c r="B28" s="60" t="s">
         <v>607</v>
@@ -9995,7 +10010,7 @@
       <c r="Q28" s="62"/>
       <c r="R28" s="62"/>
     </row>
-    <row r="29" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A29" s="53" t="s">
         <v>537</v>
       </c>
@@ -10019,7 +10034,7 @@
       <c r="Q29" s="56"/>
       <c r="R29" s="56"/>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:18" ns3:dyDescent="0.2">
       <c r="A30" s="11"/>
       <c r="B30" s="17" t="s">
         <v>611</v>
@@ -10038,7 +10053,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:18" ns3:dyDescent="0.2">
       <c r="A31" s="60"/>
       <c r="B31" s="60" t="s">
         <v>614</v>
@@ -10068,7 +10083,7 @@
       <c r="Q31" s="62"/>
       <c r="R31" s="62"/>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:18" ns3:dyDescent="0.2">
       <c r="A32" s="60"/>
       <c r="B32" s="60" t="s">
         <v>617</v>
@@ -10098,7 +10113,7 @@
       <c r="Q32" s="62"/>
       <c r="R32" s="62"/>
     </row>
-    <row r="33" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A33" s="60"/>
       <c r="B33" s="60" t="s">
         <v>620</v>
@@ -10128,7 +10143,7 @@
       <c r="Q33" s="62"/>
       <c r="R33" s="62"/>
     </row>
-    <row r="34" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A34" s="63"/>
       <c r="B34" s="63" t="s">
         <v>623</v>
@@ -10158,7 +10173,7 @@
       <c r="Q34" s="65"/>
       <c r="R34" s="65"/>
     </row>
-    <row r="35" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A35" s="63"/>
       <c r="B35" s="63" t="s">
         <v>626</v>
@@ -10188,7 +10203,7 @@
       <c r="Q35" s="65"/>
       <c r="R35" s="65"/>
     </row>
-    <row r="36" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A36" s="60"/>
       <c r="B36" s="60" t="s">
         <v>629</v>
@@ -10218,7 +10233,7 @@
       <c r="Q36" s="62"/>
       <c r="R36" s="62"/>
     </row>
-    <row r="37" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A37" s="60"/>
       <c r="B37" s="60" t="s">
         <v>632</v>
@@ -10248,7 +10263,7 @@
       <c r="Q37" s="62"/>
       <c r="R37" s="62"/>
     </row>
-    <row r="38" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A38" s="53" t="s">
         <v>537</v>
       </c>
@@ -10272,7 +10287,7 @@
       <c r="Q38" s="56"/>
       <c r="R38" s="56"/>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:18" ns3:dyDescent="0.2">
       <c r="B39" s="11" t="s">
         <v>636</v>
       </c>
@@ -10292,7 +10307,7 @@
       <c r="I39" s="11"/>
       <c r="J39" s="3"/>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:18" ns3:dyDescent="0.2">
       <c r="A40" s="60"/>
       <c r="B40" s="60" t="s">
         <v>639</v>
@@ -10322,7 +10337,7 @@
       <c r="Q40" s="62"/>
       <c r="R40" s="62"/>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:18" ns3:dyDescent="0.2">
       <c r="A41" s="60"/>
       <c r="B41" s="60" t="s">
         <v>642</v>
@@ -10352,7 +10367,7 @@
       <c r="Q41" s="62"/>
       <c r="R41" s="62"/>
     </row>
-    <row r="42" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A42" s="60"/>
       <c r="B42" s="60" t="s">
         <v>645</v>
@@ -10382,7 +10397,7 @@
       <c r="Q42" s="62"/>
       <c r="R42" s="62"/>
     </row>
-    <row r="43" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A43" s="53" t="s">
         <v>537</v>
       </c>
@@ -10406,7 +10421,7 @@
       <c r="Q43" s="56"/>
       <c r="R43" s="56"/>
     </row>
-    <row r="44" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A44" s="11"/>
       <c r="B44" s="17" t="s">
         <v>649</v>
@@ -10436,7 +10451,7 @@
       <c r="Q44" s="3"/>
       <c r="R44" s="3"/>
     </row>
-    <row r="45" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A45" s="11"/>
       <c r="B45" s="17" t="s">
         <v>652</v>
@@ -10466,7 +10481,7 @@
       <c r="Q45" s="3"/>
       <c r="R45" s="3"/>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:18" ns3:dyDescent="0.2">
       <c r="A46" s="53" t="s">
         <v>537</v>
       </c>
@@ -10490,7 +10505,7 @@
       <c r="Q46" s="56"/>
       <c r="R46" s="56"/>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:18" ns3:dyDescent="0.2">
       <c r="B47" s="11" t="s">
         <v>656</v>
       </c>
@@ -10508,7 +10523,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:18" ns3:dyDescent="0.2">
       <c r="A48" s="11"/>
       <c r="B48" s="17" t="s">
         <v>659</v>
@@ -10527,7 +10542,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A49" s="11"/>
       <c r="B49" s="17" t="s">
         <v>662</v>
@@ -10546,7 +10561,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="50" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A50" s="60"/>
       <c r="B50" s="60" t="s">
         <v>665</v>
@@ -10576,7 +10591,7 @@
       <c r="Q50" s="62"/>
       <c r="R50" s="62"/>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:18" ns3:dyDescent="0.2">
       <c r="A51" s="60"/>
       <c r="B51" s="60" t="s">
         <v>668</v>
@@ -10606,7 +10621,7 @@
       <c r="Q51" s="62"/>
       <c r="R51" s="62"/>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:18" ns3:dyDescent="0.2">
       <c r="A52" s="60"/>
       <c r="B52" s="60" t="s">
         <v>671</v>
@@ -10636,7 +10651,7 @@
       <c r="Q52" s="62"/>
       <c r="R52" s="62"/>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:18" ns3:dyDescent="0.2">
       <c r="A53" s="60"/>
       <c r="B53" s="60" t="s">
         <v>674</v>
@@ -10666,7 +10681,7 @@
       <c r="Q53" s="62"/>
       <c r="R53" s="62"/>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:18" ns3:dyDescent="0.2">
       <c r="A54" s="62"/>
       <c r="B54" s="60" t="s">
         <v>677</v>
@@ -10696,7 +10711,7 @@
       <c r="Q54" s="62"/>
       <c r="R54" s="62"/>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:18" ns3:dyDescent="0.2">
       <c r="A55" s="60"/>
       <c r="B55" s="60" t="s">
         <v>680</v>
@@ -10726,7 +10741,7 @@
       <c r="Q55" s="62"/>
       <c r="R55" s="62"/>
     </row>
-    <row r="56" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A56" s="60"/>
       <c r="B56" s="60" t="s">
         <v>683</v>
@@ -10756,7 +10771,7 @@
       <c r="Q56" s="62"/>
       <c r="R56" s="62"/>
     </row>
-    <row r="57" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A57" s="60"/>
       <c r="B57" s="60" t="s">
         <v>686</v>
@@ -10786,7 +10801,7 @@
       <c r="Q57" s="62"/>
       <c r="R57" s="62"/>
     </row>
-    <row r="58" spans="1:18" ht="18.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:18" ht="18.95" customHeight="1" ns3:dyDescent="0.2">
       <c r="A58" s="60"/>
       <c r="B58" s="60" t="s">
         <v>689</v>
@@ -10816,7 +10831,7 @@
       <c r="Q58" s="62"/>
       <c r="R58" s="62"/>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:18" ns3:dyDescent="0.2">
       <c r="A59" s="53" t="s">
         <v>537</v>
       </c>
@@ -10840,7 +10855,7 @@
       <c r="Q59" s="56"/>
       <c r="R59" s="56"/>
     </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:18" ns3:dyDescent="0.2">
       <c r="A60" s="60"/>
       <c r="B60" s="60" t="s">
         <v>693</v>
@@ -10870,7 +10885,7 @@
       <c r="Q60" s="62"/>
       <c r="R60" s="62"/>
     </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:18" ns3:dyDescent="0.2">
       <c r="A61" s="11"/>
       <c r="B61" s="11"/>
       <c r="C61" s="11"/>
@@ -10879,7 +10894,7 @@
       <c r="F61" s="11"/>
       <c r="G61" s="11"/>
     </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:18" ns3:dyDescent="0.2">
       <c r="A62" s="11"/>
       <c r="B62" s="11"/>
       <c r="C62" s="11"/>
@@ -10888,7 +10903,7 @@
       <c r="F62" s="11"/>
       <c r="G62" s="11"/>
     </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:18" ns3:dyDescent="0.2">
       <c r="A63" s="11"/>
       <c r="B63" s="11"/>
       <c r="C63" s="11"/>
@@ -10897,7 +10912,7 @@
       <c r="F63" s="11"/>
       <c r="G63" s="11"/>
     </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:18" ns3:dyDescent="0.2">
       <c r="A64" s="11"/>
       <c r="B64" s="11"/>
       <c r="C64" s="11"/>
@@ -10906,7 +10921,7 @@
       <c r="F64" s="11"/>
       <c r="G64" s="11"/>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:7" ns3:dyDescent="0.2">
       <c r="A65" s="11"/>
       <c r="B65" s="11"/>
       <c r="C65" s="11"/>
@@ -10915,7 +10930,7 @@
       <c r="F65" s="11"/>
       <c r="G65" s="11"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:7" ns3:dyDescent="0.2">
       <c r="A73" s="11"/>
       <c r="B73" s="11"/>
       <c r="C73" s="11"/>
@@ -10924,7 +10939,7 @@
       <c r="F73" s="11"/>
       <c r="G73" s="11"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:7" ns3:dyDescent="0.2">
       <c r="A74" s="11"/>
       <c r="B74" s="11"/>
       <c r="C74" s="11"/>
@@ -10933,7 +10948,7 @@
       <c r="F74" s="11"/>
       <c r="G74" s="11"/>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:7" ns3:dyDescent="0.2">
       <c r="A75" s="11"/>
       <c r="B75" s="11"/>
       <c r="C75" s="11"/>
@@ -10942,7 +10957,7 @@
       <c r="F75" s="11"/>
       <c r="G75" s="11"/>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:7" ns3:dyDescent="0.2">
       <c r="A76" s="11"/>
       <c r="B76" s="11"/>
       <c r="C76" s="11"/>
@@ -10951,7 +10966,7 @@
       <c r="F76" s="11"/>
       <c r="G76" s="11"/>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:7" ns3:dyDescent="0.2">
       <c r="A77" s="11"/>
       <c r="B77" s="11"/>
       <c r="C77" s="11"/>
@@ -10960,7 +10975,7 @@
       <c r="F77" s="11"/>
       <c r="G77" s="11"/>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:7" ns3:dyDescent="0.2">
       <c r="A78" s="11"/>
       <c r="B78" s="11"/>
       <c r="C78" s="11"/>
@@ -10969,7 +10984,7 @@
       <c r="F78" s="11"/>
       <c r="G78" s="11"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:7" ns3:dyDescent="0.2">
       <c r="A79" s="11"/>
       <c r="B79" s="11"/>
       <c r="C79" s="11"/>
@@ -10978,7 +10993,7 @@
       <c r="F79" s="11"/>
       <c r="G79" s="11"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:7" ns3:dyDescent="0.2">
       <c r="A80" s="11"/>
       <c r="B80" s="11"/>
       <c r="C80" s="11"/>
@@ -10987,7 +11002,7 @@
       <c r="F80" s="11"/>
       <c r="G80" s="11"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:7" ns3:dyDescent="0.2">
       <c r="A81" s="11"/>
       <c r="B81" s="11"/>
       <c r="C81" s="11"/>
@@ -10996,7 +11011,7 @@
       <c r="F81" s="11"/>
       <c r="G81" s="11"/>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:7" ns3:dyDescent="0.2">
       <c r="A82" s="11"/>
       <c r="B82" s="11"/>
       <c r="C82" s="11"/>
@@ -11005,7 +11020,7 @@
       <c r="F82" s="11"/>
       <c r="G82" s="11"/>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:7" ns3:dyDescent="0.2">
       <c r="A83" s="11"/>
       <c r="B83" s="11"/>
       <c r="C83" s="11"/>
@@ -11014,7 +11029,7 @@
       <c r="F83" s="11"/>
       <c r="G83" s="11"/>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:7" ns3:dyDescent="0.2">
       <c r="A84" s="11"/>
       <c r="B84" s="11"/>
       <c r="C84" s="11"/>
@@ -11023,7 +11038,7 @@
       <c r="F84" s="11"/>
       <c r="G84" s="11"/>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:7" ns3:dyDescent="0.2">
       <c r="A85" s="11"/>
       <c r="B85" s="11"/>
       <c r="C85" s="11"/>
@@ -11032,7 +11047,7 @@
       <c r="F85" s="11"/>
       <c r="G85" s="11"/>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:7" ns3:dyDescent="0.2">
       <c r="A86" s="11"/>
       <c r="B86" s="11"/>
       <c r="C86" s="11"/>
@@ -11041,7 +11056,7 @@
       <c r="F86" s="11"/>
       <c r="G86" s="11"/>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:7" ns3:dyDescent="0.2">
       <c r="A87" s="11"/>
       <c r="B87" s="11"/>
       <c r="C87" s="11"/>
@@ -11050,7 +11065,7 @@
       <c r="F87" s="11"/>
       <c r="G87" s="11"/>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:7" ns3:dyDescent="0.2">
       <c r="A88" s="11"/>
       <c r="B88" s="11"/>
       <c r="C88" s="11"/>
@@ -11059,7 +11074,7 @@
       <c r="F88" s="11"/>
       <c r="G88" s="11"/>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:7" ns3:dyDescent="0.2">
       <c r="A89" s="11"/>
       <c r="B89" s="11"/>
       <c r="C89" s="11"/>
@@ -11068,7 +11083,7 @@
       <c r="F89" s="11"/>
       <c r="G89" s="11"/>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:7" ns3:dyDescent="0.2">
       <c r="A90" s="11"/>
       <c r="B90" s="11"/>
       <c r="C90" s="11"/>
@@ -11077,7 +11092,7 @@
       <c r="F90" s="11"/>
       <c r="G90" s="11"/>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:7" ns3:dyDescent="0.2">
       <c r="A91" s="11"/>
       <c r="B91" s="11"/>
       <c r="C91" s="11"/>
@@ -11086,7 +11101,7 @@
       <c r="F91" s="11"/>
       <c r="G91" s="11"/>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:7" ns3:dyDescent="0.2">
       <c r="A92" s="11"/>
       <c r="B92" s="11"/>
       <c r="C92" s="11"/>
@@ -11095,7 +11110,7 @@
       <c r="F92" s="11"/>
       <c r="G92" s="11"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:7" ns3:dyDescent="0.2">
       <c r="A93" s="11"/>
       <c r="B93" s="11"/>
       <c r="C93" s="11"/>
@@ -11104,7 +11119,7 @@
       <c r="F93" s="11"/>
       <c r="G93" s="11"/>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:7" ns3:dyDescent="0.2">
       <c r="A94" s="11"/>
       <c r="B94" s="11"/>
       <c r="C94" s="11"/>
@@ -11113,7 +11128,7 @@
       <c r="F94" s="11"/>
       <c r="G94" s="11"/>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:7" ns3:dyDescent="0.2">
       <c r="A95" s="11"/>
       <c r="B95" s="11"/>
       <c r="C95" s="11"/>
@@ -11122,7 +11137,7 @@
       <c r="F95" s="11"/>
       <c r="G95" s="11"/>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:7" ns3:dyDescent="0.2">
       <c r="A96" s="11"/>
       <c r="B96" s="11"/>
       <c r="C96" s="11"/>
@@ -11131,7 +11146,7 @@
       <c r="F96" s="11"/>
       <c r="G96" s="11"/>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:7" ns3:dyDescent="0.2">
       <c r="A97" s="11"/>
       <c r="B97" s="11"/>
       <c r="C97" s="11"/>
@@ -11140,7 +11155,7 @@
       <c r="F97" s="11"/>
       <c r="G97" s="11"/>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:7" ns3:dyDescent="0.2">
       <c r="A98" s="11"/>
       <c r="B98" s="11"/>
       <c r="C98" s="11"/>
@@ -11149,7 +11164,7 @@
       <c r="F98" s="11"/>
       <c r="G98" s="11"/>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:7" ns3:dyDescent="0.2">
       <c r="A99" s="11"/>
       <c r="B99" s="11"/>
       <c r="C99" s="11"/>
@@ -11158,7 +11173,7 @@
       <c r="F99" s="11"/>
       <c r="G99" s="11"/>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:7" ns3:dyDescent="0.2">
       <c r="A100" s="11"/>
       <c r="B100" s="11"/>
       <c r="C100" s="11"/>
@@ -11167,7 +11182,7 @@
       <c r="F100" s="11"/>
       <c r="G100" s="11"/>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:7" ns3:dyDescent="0.2">
       <c r="A101" s="11"/>
       <c r="B101" s="11"/>
       <c r="C101" s="11"/>
@@ -11176,7 +11191,7 @@
       <c r="F101" s="11"/>
       <c r="G101" s="11"/>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:7" ns3:dyDescent="0.2">
       <c r="A102" s="11"/>
       <c r="B102" s="11"/>
       <c r="C102" s="11"/>
@@ -11185,7 +11200,7 @@
       <c r="F102" s="11"/>
       <c r="G102" s="11"/>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:7" ns3:dyDescent="0.2">
       <c r="A103" s="11"/>
       <c r="B103" s="11"/>
       <c r="C103" s="11"/>
@@ -11194,7 +11209,7 @@
       <c r="F103" s="11"/>
       <c r="G103" s="11"/>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:7" ns3:dyDescent="0.2">
       <c r="A104" s="11"/>
       <c r="B104" s="11"/>
       <c r="C104" s="11"/>
@@ -11203,7 +11218,7 @@
       <c r="F104" s="11"/>
       <c r="G104" s="11"/>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:7" ns3:dyDescent="0.2">
       <c r="A105" s="11"/>
       <c r="B105" s="11"/>
       <c r="C105" s="11"/>
@@ -11212,7 +11227,7 @@
       <c r="F105" s="11"/>
       <c r="G105" s="11"/>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:7" ns3:dyDescent="0.2">
       <c r="A106" s="11"/>
       <c r="B106" s="11"/>
       <c r="C106" s="11"/>
@@ -11221,7 +11236,7 @@
       <c r="F106" s="11"/>
       <c r="G106" s="11"/>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:7" ns3:dyDescent="0.2">
       <c r="A107" s="11"/>
       <c r="B107" s="11"/>
       <c r="C107" s="11"/>
@@ -11230,7 +11245,7 @@
       <c r="F107" s="11"/>
       <c r="G107" s="11"/>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:7" ns3:dyDescent="0.2">
       <c r="A108" s="11"/>
       <c r="B108" s="11"/>
       <c r="C108" s="11"/>
@@ -11239,7 +11254,7 @@
       <c r="F108" s="11"/>
       <c r="G108" s="11"/>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:7" ns3:dyDescent="0.2">
       <c r="A109" s="11"/>
       <c r="B109" s="11"/>
       <c r="C109" s="11"/>
@@ -11248,7 +11263,7 @@
       <c r="F109" s="11"/>
       <c r="G109" s="11"/>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:7" ns3:dyDescent="0.2">
       <c r="A110" s="11"/>
       <c r="B110" s="11"/>
       <c r="C110" s="11"/>
@@ -11257,7 +11272,7 @@
       <c r="F110" s="11"/>
       <c r="G110" s="11"/>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:7" ns3:dyDescent="0.2">
       <c r="A111" s="11"/>
       <c r="B111" s="11"/>
       <c r="C111" s="11"/>
@@ -11266,7 +11281,7 @@
       <c r="F111" s="11"/>
       <c r="G111" s="11"/>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:7" ns3:dyDescent="0.2">
       <c r="A112" s="11"/>
       <c r="B112" s="11"/>
       <c r="C112" s="11"/>
@@ -11275,7 +11290,7 @@
       <c r="F112" s="11"/>
       <c r="G112" s="11"/>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:7" ns3:dyDescent="0.2">
       <c r="A113" s="11"/>
       <c r="B113" s="11"/>
       <c r="C113" s="11"/>
@@ -11284,7 +11299,7 @@
       <c r="F113" s="11"/>
       <c r="G113" s="11"/>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:7" ns3:dyDescent="0.2">
       <c r="A114" s="11"/>
       <c r="B114" s="11"/>
       <c r="C114" s="11"/>
@@ -11293,7 +11308,7 @@
       <c r="F114" s="11"/>
       <c r="G114" s="11"/>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:7" ns3:dyDescent="0.2">
       <c r="A115" s="11"/>
       <c r="B115" s="11"/>
       <c r="C115" s="11"/>
@@ -11302,7 +11317,7 @@
       <c r="F115" s="11"/>
       <c r="G115" s="11"/>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:7" ns3:dyDescent="0.2">
       <c r="A116" s="11"/>
       <c r="B116" s="11"/>
       <c r="C116" s="11"/>
@@ -11311,7 +11326,7 @@
       <c r="F116" s="11"/>
       <c r="G116" s="11"/>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:7" ns3:dyDescent="0.2">
       <c r="A117" s="11"/>
       <c r="B117" s="11"/>
       <c r="C117" s="11"/>
@@ -11320,7 +11335,7 @@
       <c r="F117" s="11"/>
       <c r="G117" s="11"/>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:7" ns3:dyDescent="0.2">
       <c r="A118" s="11"/>
       <c r="B118" s="11"/>
       <c r="C118" s="11"/>
@@ -11329,7 +11344,7 @@
       <c r="F118" s="11"/>
       <c r="G118" s="11"/>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:7" ns3:dyDescent="0.2">
       <c r="A119" s="11"/>
       <c r="B119" s="11"/>
       <c r="C119" s="11"/>
@@ -11338,7 +11353,7 @@
       <c r="F119" s="11"/>
       <c r="G119" s="11"/>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:7" ns3:dyDescent="0.2">
       <c r="A120" s="11"/>
       <c r="B120" s="11"/>
       <c r="C120" s="11"/>
@@ -11347,7 +11362,7 @@
       <c r="F120" s="11"/>
       <c r="G120" s="11"/>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:7" ns3:dyDescent="0.2">
       <c r="A121" s="11"/>
       <c r="B121" s="11"/>
       <c r="C121" s="11"/>
@@ -11356,7 +11371,7 @@
       <c r="F121" s="11"/>
       <c r="G121" s="11"/>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:7" ns3:dyDescent="0.2">
       <c r="A122" s="11"/>
       <c r="B122" s="11"/>
       <c r="C122" s="11"/>
@@ -11365,7 +11380,7 @@
       <c r="F122" s="11"/>
       <c r="G122" s="11"/>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:7" ns3:dyDescent="0.2">
       <c r="A123" s="11"/>
       <c r="B123" s="11"/>
       <c r="C123" s="11"/>
@@ -11374,7 +11389,7 @@
       <c r="F123" s="11"/>
       <c r="G123" s="11"/>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:7" ns3:dyDescent="0.2">
       <c r="A124" s="11"/>
       <c r="B124" s="11"/>
       <c r="C124" s="11"/>
@@ -11383,7 +11398,7 @@
       <c r="F124" s="11"/>
       <c r="G124" s="11"/>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:7" ns3:dyDescent="0.2">
       <c r="A125" s="11"/>
       <c r="B125" s="11"/>
       <c r="C125" s="11"/>
@@ -11392,7 +11407,7 @@
       <c r="F125" s="11"/>
       <c r="G125" s="11"/>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:7" ns3:dyDescent="0.2">
       <c r="A126" s="11"/>
       <c r="B126" s="11"/>
       <c r="C126" s="11"/>
@@ -11401,7 +11416,7 @@
       <c r="F126" s="11"/>
       <c r="G126" s="11"/>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:7" ns3:dyDescent="0.2">
       <c r="A127" s="11"/>
       <c r="B127" s="11"/>
       <c r="C127" s="11"/>
@@ -11410,7 +11425,7 @@
       <c r="F127" s="11"/>
       <c r="G127" s="11"/>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:7" ns3:dyDescent="0.2">
       <c r="A128" s="11"/>
       <c r="B128" s="11"/>
       <c r="C128" s="11"/>
@@ -11419,7 +11434,7 @@
       <c r="F128" s="11"/>
       <c r="G128" s="11"/>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:7" ns3:dyDescent="0.2">
       <c r="A129" s="11"/>
       <c r="B129" s="11"/>
       <c r="C129" s="11"/>
@@ -11428,7 +11443,7 @@
       <c r="F129" s="11"/>
       <c r="G129" s="11"/>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:7" ns3:dyDescent="0.2">
       <c r="A130" s="11"/>
       <c r="B130" s="11"/>
       <c r="C130" s="11"/>
@@ -11437,7 +11452,7 @@
       <c r="F130" s="11"/>
       <c r="G130" s="11"/>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:7" ns3:dyDescent="0.2">
       <c r="A131" s="11"/>
       <c r="B131" s="11"/>
       <c r="C131" s="11"/>
@@ -11446,7 +11461,7 @@
       <c r="F131" s="11"/>
       <c r="G131" s="11"/>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:7" ns3:dyDescent="0.2">
       <c r="A132" s="11"/>
       <c r="B132" s="11"/>
       <c r="C132" s="11"/>
@@ -11455,7 +11470,7 @@
       <c r="F132" s="11"/>
       <c r="G132" s="11"/>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:7" ns3:dyDescent="0.2">
       <c r="A133" s="11"/>
       <c r="B133" s="11"/>
       <c r="C133" s="11"/>
@@ -11464,7 +11479,7 @@
       <c r="F133" s="11"/>
       <c r="G133" s="11"/>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:7" ns3:dyDescent="0.2">
       <c r="A134" s="11"/>
       <c r="B134" s="11"/>
       <c r="C134" s="11"/>
@@ -11473,7 +11488,7 @@
       <c r="F134" s="11"/>
       <c r="G134" s="11"/>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:7" ns3:dyDescent="0.2">
       <c r="A135" s="11"/>
       <c r="B135" s="11"/>
       <c r="C135" s="11"/>
@@ -11482,7 +11497,7 @@
       <c r="F135" s="11"/>
       <c r="G135" s="11"/>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:7" ns3:dyDescent="0.2">
       <c r="A136" s="11"/>
       <c r="B136" s="11"/>
       <c r="C136" s="11"/>
@@ -11491,7 +11506,7 @@
       <c r="F136" s="11"/>
       <c r="G136" s="11"/>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:7" ns3:dyDescent="0.2">
       <c r="A137" s="11"/>
       <c r="B137" s="11"/>
       <c r="C137" s="11"/>
@@ -11500,7 +11515,7 @@
       <c r="F137" s="11"/>
       <c r="G137" s="11"/>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:7" ns3:dyDescent="0.2">
       <c r="A138" s="11"/>
       <c r="B138" s="11"/>
       <c r="C138" s="11"/>
@@ -11509,7 +11524,7 @@
       <c r="F138" s="11"/>
       <c r="G138" s="11"/>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:7" ns3:dyDescent="0.2">
       <c r="A139" s="11"/>
       <c r="B139" s="11"/>
       <c r="C139" s="11"/>
@@ -11518,7 +11533,7 @@
       <c r="F139" s="11"/>
       <c r="G139" s="11"/>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:7" ns3:dyDescent="0.2">
       <c r="A140" s="11"/>
       <c r="B140" s="11"/>
       <c r="C140" s="11"/>
@@ -11527,7 +11542,7 @@
       <c r="F140" s="11"/>
       <c r="G140" s="11"/>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:7" ns3:dyDescent="0.2">
       <c r="A141" s="11"/>
       <c r="B141" s="11"/>
       <c r="C141" s="11"/>
@@ -11536,7 +11551,7 @@
       <c r="F141" s="11"/>
       <c r="G141" s="11"/>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:7" ns3:dyDescent="0.2">
       <c r="A142" s="11"/>
       <c r="B142" s="11"/>
       <c r="C142" s="11"/>
@@ -11545,7 +11560,7 @@
       <c r="F142" s="11"/>
       <c r="G142" s="11"/>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:7" ns3:dyDescent="0.2">
       <c r="A143" s="11"/>
       <c r="B143" s="11"/>
       <c r="C143" s="11"/>
@@ -11554,7 +11569,7 @@
       <c r="F143" s="11"/>
       <c r="G143" s="11"/>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:7" ns3:dyDescent="0.2">
       <c r="A144" s="11"/>
       <c r="B144" s="11"/>
       <c r="C144" s="11"/>
@@ -11563,7 +11578,7 @@
       <c r="F144" s="11"/>
       <c r="G144" s="11"/>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:7" ns3:dyDescent="0.2">
       <c r="A145" s="11"/>
       <c r="B145" s="11"/>
       <c r="C145" s="11"/>
@@ -11572,7 +11587,7 @@
       <c r="F145" s="11"/>
       <c r="G145" s="11"/>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:7" ns3:dyDescent="0.2">
       <c r="A146" s="11"/>
       <c r="B146" s="11"/>
       <c r="C146" s="11"/>
@@ -11581,7 +11596,7 @@
       <c r="F146" s="11"/>
       <c r="G146" s="11"/>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:7" ns3:dyDescent="0.2">
       <c r="A147" s="11"/>
       <c r="B147" s="11"/>
       <c r="C147" s="11"/>
@@ -11590,7 +11605,7 @@
       <c r="F147" s="11"/>
       <c r="G147" s="11"/>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:7" ns3:dyDescent="0.2">
       <c r="A148" s="11"/>
       <c r="B148" s="11"/>
       <c r="C148" s="11"/>
@@ -11599,7 +11614,7 @@
       <c r="F148" s="11"/>
       <c r="G148" s="11"/>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:7" ns3:dyDescent="0.2">
       <c r="A149" s="11"/>
       <c r="B149" s="11"/>
       <c r="C149" s="11"/>
@@ -11611,8 +11626,8 @@
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <drawing ns4:id="rId1"/>
+  <legacyDrawing ns4:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: migrate record references to typed keys
</commit_message>
<xml_diff>
--- a/examples/humanpark/data/Configs.xlsx
+++ b/examples/humanpark/data/Configs.xlsx
@@ -2651,19 +2651,19 @@
     <t>Gene_LingHuoE|Gene_FaGuangQi</t>
   </si>
   <si>
-    <t>@Gene_SimpleDivision|@Gene_Chloroplast|@Gene_Flagellum|@Gene_LvShi</t>
-  </si>
-  <si>
-    <t>@Gene_LingHuoE|@Gene_FaGuangQi</t>
-  </si>
-  <si>
-    <t>@Gene_TanHuangJiRou</t>
-  </si>
-  <si>
-    <t>@Gene_DuCiXiBao</t>
-  </si>
-  <si>
-    <t>@Gene_Genius</t>
+    <t>@GeneConfig.Gene_SimpleDivision|@GeneConfig.Gene_Chloroplast|@GeneConfig.Gene_Flagellum|@GeneConfig.Gene_LvShi</t>
+  </si>
+  <si>
+    <t>@GeneConfig.Gene_LingHuoE|@GeneConfig.Gene_FaGuangQi</t>
+  </si>
+  <si>
+    <t>@GeneConfig.Gene_TanHuangJiRou</t>
+  </si>
+  <si>
+    <t>@GeneConfig.Gene_DuCiXiBao</t>
+  </si>
+  <si>
+    <t>@GeneConfig.Gene_Genius</t>
   </si>
 </sst>
 </file>

</xml_diff>